<commit_message>
Strengthen seeded defect detection audit
</commit_message>
<xml_diff>
--- a/reports/defect_detection_summary.xlsx
+++ b/reports/defect_detection_summary.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Defect_Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Validation_Findings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,10 +436,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Expected_Keywords</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Match_Count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Matched_Finding</t>
         </is>
@@ -462,12 +473,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>CT005 | Age is missing</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-002 | Participant CT005: Age is missing or not an integer.</t>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Participant CT005: Age is missing or not an integer.</t>
         </is>
       </c>
     </row>
@@ -489,12 +508,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>duplicate Subject_ID CT005</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-001 | Participants: duplicate Subject_ID CT005.</t>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Participants: duplicate Subject_ID CT005.</t>
         </is>
       </c>
     </row>
@@ -516,12 +543,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Visit row 12 | Visit_Date</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-009 | Visit row 12: missing or invalid Visit_Date.</t>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Visit row 12: missing or invalid Visit_Date.</t>
         </is>
       </c>
     </row>
@@ -543,12 +578,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>CT007 Week 4 | Day 40</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>REVIEW | VAL-012 | CT007 Week 4 is Day 40; expected Days 21-35.</t>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CT007 Week 4 is Day 40; expected Days 21-35.</t>
         </is>
       </c>
     </row>
@@ -570,12 +613,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>Lab row 6 | CT999</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-013 | Lab row 6: unknown or missing subject 'CT999'.</t>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lab row 6: unknown or missing subject 'CT999'.</t>
         </is>
       </c>
     </row>
@@ -597,12 +648,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>duplicate Lab_ID LAB006</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-028 | Laboratory: duplicate Lab_ID LAB006.</t>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Laboratory: duplicate Lab_ID LAB006.</t>
         </is>
       </c>
     </row>
@@ -624,12 +683,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Lab row 8 | mg/L</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-017 | Lab row 8: invalid Unit 'mg/L'.</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Lab row 8: invalid Unit 'mg/L'.</t>
         </is>
       </c>
     </row>
@@ -651,12 +718,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Lab row 9 | non-numeric</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-016 | Lab row 9: result is missing, non-numeric, or not positive.</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Lab row 9: result is missing, non-numeric, or not positive.</t>
         </is>
       </c>
     </row>
@@ -678,12 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>LAB023 | Missed</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-020 | LAB023: laboratory record is linked to a visit with status 'Missed'.</t>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>LAB023: laboratory record is linked to a visit with status 'Missed'.</t>
         </is>
       </c>
     </row>
@@ -705,12 +788,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>AE001 | before consent</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>REVIEW | VAL-025 | AE AE001: onset date is before consent date.</t>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AE AE001: onset date is before consent date.</t>
         </is>
       </c>
     </row>
@@ -732,12 +823,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>CT010 Baseline | Day -1</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>REVIEW | VAL-012 | CT010 Baseline is Day -1; expected Day 0.</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CT010 Baseline is Day -1; expected Day 0.</t>
         </is>
       </c>
     </row>
@@ -759,12 +858,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>AE row 13 | CT999</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ERROR | VAL-022 | AE row 13: unknown or missing subject 'CT999'.</t>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>AE row 13: unknown or missing subject 'CT999'.</t>
         </is>
       </c>
     </row>
@@ -807,4 +914,443 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Finding_Type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Rule_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Finding_Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VAL-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Participants: duplicate Subject_ID CT005.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VAL-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Participant CT005: Age is missing or not an integer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VAL-007</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Visit row 17: subject 'CT006' does not exist in Participants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VAL-007</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Visit row 18: subject 'CT006' does not exist in Participants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VAL-007</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Visit row 19: subject 'CT006' does not exist in Participants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VAL-009</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Visit row 12: missing or invalid Visit_Date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VAL-013</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lab row 6: unknown or missing subject 'CT999'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>VAL-013</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lab row 17: unknown or missing subject 'CT006'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>VAL-013</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lab row 18: unknown or missing subject 'CT006'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>VAL-013</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lab row 19: unknown or missing subject 'CT006'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VAL-016</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Lab row 9: result is missing, non-numeric, or not positive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>VAL-017</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lab row 8: invalid Unit 'mg/L'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>VAL-020</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LAB005: no matching visit for CT999 / Week 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VAL-020</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LAB011: no matching visit for CT004 / Week 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>VAL-020</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LAB023: laboratory record is linked to a visit with status 'Missed'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VAL-028</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Laboratory: duplicate Lab_ID LAB006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VAL-028</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Duplicate measurement: CT002 / Week 8 / Glucose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VAL-028</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Duplicate measurement: CT002 / Week 8 / Glucose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VAL-022</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AE row 13: unknown or missing subject 'CT999'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VAL-012</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CT007 Week 4 is Day 40; expected Days 21-35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VAL-012</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CT010 Baseline is Day -1; expected Day 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>VAL-021</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>LAB020: Collection_Date differs from the matching visit date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>VAL-021</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LAB028: Collection_Date differs from the matching visit date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>VAL-025</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AE AE001: onset date is before consent date.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>